<commit_message>
added test scenrario in comment
</commit_message>
<xml_diff>
--- a/WorkShopDemo/TestData/TestScriptData.xlsx
+++ b/WorkShopDemo/TestData/TestScriptData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Premshankar Mishra\Git\TP\Selenium\April_8\8_April\TestData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Premshankar Mishra\Git\TP\Selenium\WorkShopDemo\WorkShopDemo\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5865884C-9674-48B3-918C-3320852F366B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" tabRatio="500" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2988" yWindow="2100" windowWidth="17280" windowHeight="8880" tabRatio="500" firstSheet="6" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="org" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="151">
   <si>
     <t>TC_ID</t>
   </si>
@@ -469,37 +469,31 @@
     <t>orderDetails</t>
   </si>
   <si>
-    <t>2267247</t>
-  </si>
-  <si>
-    <t>2267248</t>
-  </si>
-  <si>
     <t>Order number:</t>
   </si>
   <si>
-    <t>2267256</t>
-  </si>
-  <si>
-    <t>2267257</t>
-  </si>
-  <si>
-    <t>2267258</t>
-  </si>
-  <si>
-    <t>2267259</t>
-  </si>
-  <si>
-    <t>2267260</t>
-  </si>
-  <si>
-    <t>2267261</t>
-  </si>
-  <si>
-    <t>2267374</t>
-  </si>
-  <si>
-    <t>2267375</t>
+    <t>2267456</t>
+  </si>
+  <si>
+    <t>2267457</t>
+  </si>
+  <si>
+    <t>2267458</t>
+  </si>
+  <si>
+    <t>2267459</t>
+  </si>
+  <si>
+    <t>2267462</t>
+  </si>
+  <si>
+    <t>2267463</t>
+  </si>
+  <si>
+    <t>2267466</t>
+  </si>
+  <si>
+    <t>2267467</t>
   </si>
 </sst>
 </file>
@@ -1198,7 +1192,7 @@
         <v>141</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2082,10 +2076,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed useless wait commands
</commit_message>
<xml_diff>
--- a/WorkShopDemo/TestData/TestScriptData.xlsx
+++ b/WorkShopDemo/TestData/TestScriptData.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="155">
   <si>
     <t>TC_ID</t>
   </si>
@@ -494,6 +494,18 @@
   </si>
   <si>
     <t>2267467</t>
+  </si>
+  <si>
+    <t>2267484</t>
+  </si>
+  <si>
+    <t>2267485</t>
+  </si>
+  <si>
+    <t>2267487</t>
+  </si>
+  <si>
+    <t>2267488</t>
   </si>
 </sst>
 </file>
@@ -2076,10 +2088,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B2" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added print stmnt and comment
</commit_message>
<xml_diff>
--- a/WorkShopDemo/TestData/TestScriptData.xlsx
+++ b/WorkShopDemo/TestData/TestScriptData.xlsx
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="162">
   <si>
     <t>TC_ID</t>
   </si>
@@ -512,6 +512,21 @@
   </si>
   <si>
     <t>2267494</t>
+  </si>
+  <si>
+    <t>2267505</t>
+  </si>
+  <si>
+    <t>2267506</t>
+  </si>
+  <si>
+    <t>2267517</t>
+  </si>
+  <si>
+    <t>2267518</t>
+  </si>
+  <si>
+    <t>2267519</t>
   </si>
 </sst>
 </file>
@@ -2094,10 +2109,10 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>